<commit_message>
edit mapping (adapt #REC intervals & reorder Free1 commands)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping-fruits.xlsx
+++ b/inst/extdata/mapping-fruits.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="78">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -193,9 +193,30 @@
     <t xml:space="preserve">Others</t>
   </si>
   <si>
+    <t xml:space="preserve">#COMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_fruits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">((dat_mod |&gt; dplyr::select(q2_1:q2_97)) == 1) |&gt; rowSums()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#IF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_fruits == 0 &amp; q1 == 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q2_99 = 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">#VARL</t>
   </si>
   <si>
+    <t xml:space="preserve">q2_99</t>
+  </si>
+  <si>
     <t xml:space="preserve">q{2 3}_1</t>
   </si>
   <si>
@@ -208,30 +229,6 @@
     <t xml:space="preserve">q{2 3}_97</t>
   </si>
   <si>
-    <t xml:space="preserve">#COMP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n_fruits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">((dat_mod |&gt; dplyr::select(q2_1:q2_97)) == 1) |&gt; rowSums()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#IF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n_fruits == 0 &amp; q1 == 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q2_00 = 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q2_00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None selected</t>
-  </si>
-  <si>
     <t xml:space="preserve">n_fruits == 1 &amp; q2_{1 2 3 97} == 1</t>
   </si>
   <si>
@@ -247,10 +244,10 @@
     <t xml:space="preserve">Fruit number category</t>
   </si>
   <si>
-    <t xml:space="preserve">2 or less</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 or 4</t>
+    <t xml:space="preserve">3 or less</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 or 5</t>
   </si>
   <si>
     <t xml:space="preserve">.</t>
@@ -259,7 +256,7 @@
     <t xml:space="preserve">Inf</t>
   </si>
   <si>
-    <t xml:space="preserve">5 and more</t>
+    <t xml:space="preserve">6 and more</t>
   </si>
 </sst>
 </file>
@@ -349,7 +346,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -362,12 +359,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1216,157 +1217,159 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A4:E17"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A3:E17"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="29.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="30.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="3" width="8.59"/>
   </cols>
   <sheetData>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C5" s="1" t="s">
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="3" t="s">
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="1" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="1" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="1" t="n">
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="E16" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="n">
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="E17" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D17" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>